<commit_message>
Add color-trim block, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files: 12
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-bronco.report.xlsx
+++ b/tools/importer/reports/import-bronco.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="18">
   <si>
     <t>_reportFile</t>
   </si>
@@ -56,6 +56,15 @@
   </si>
   <si>
     <t>http://127.0.0.1:8765/bronco.html</t>
+  </si>
+  <si>
+    <t>innovationlabgt/bronco.report.json</t>
+  </si>
+  <si>
+    <t>innovationlabgt/bronco</t>
+  </si>
+  <si>
+    <t>2026-09-29T18:49:47.429Z</t>
   </si>
 </sst>
 </file>
@@ -444,12 +453,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="20" customWidth="1"/>
+    <col min="1" max="1" width="36" customWidth="1"/>
     <col min="2" max="2" width="50" customWidth="1"/>
-    <col min="3" max="3" width="8" customWidth="1"/>
+    <col min="3" max="3" width="24" customWidth="1"/>
     <col min="5" max="5" width="10" customWidth="1"/>
     <col min="6" max="6" width="26" customWidth="1"/>
     <col min="7" max="7" width="33" customWidth="1"/>
@@ -508,6 +517,32 @@
         <v>14</v>
       </c>
     </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3" t="s">
+        <v>17</v>
+      </c>
+      <c r="G3" t="s">
+        <v>13</v>
+      </c>
+      <c r="H3" t="s">
+        <v>14</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Add color-trim, trim-tab blocks, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files: 31
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-bronco.report.xlsx
+++ b/tools/importer/reports/import-bronco.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="19">
   <si>
     <t>_reportFile</t>
   </si>
@@ -61,10 +61,13 @@
     <t>innovationlabgt/bronco.report.json</t>
   </si>
   <si>
+    <t>["hero-vehicle","trim-tab","trim-tab","trim-tab","trim-tab","trim-tab","trim-tab","trim-tab","trim-tab","trim-tab","trim-tab","trim-tab","trim-tab","trim-tab","trim-tab","trim-tab","trim-tab","trim-tab","trim-tab","trim-tab","trim-tab","trim-tab","trim-tab","trim-tab","trim-tab"]</t>
+  </si>
+  <si>
     <t>innovationlabgt/bronco</t>
   </si>
   <si>
-    <t>2026-09-29T18:49:47.429Z</t>
+    <t>2026-09-29T20:16:57.195Z</t>
   </si>
 </sst>
 </file>
@@ -522,10 +525,10 @@
         <v>15</v>
       </c>
       <c r="B3" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="C3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D3" t="s">
         <v>11</v>
@@ -534,7 +537,7 @@
         <v>10</v>
       </c>
       <c r="F3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G3" t="s">
         <v>13</v>

</xml_diff>

<commit_message>
Add header, trim-tab blocks, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files: 22
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-bronco.report.xlsx
+++ b/tools/importer/reports/import-bronco.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="24">
   <si>
     <t>_reportFile</t>
   </si>
@@ -58,6 +58,21 @@
     <t>http://127.0.0.1:8765/bronco.html</t>
   </si>
   <si>
+    <t>nav.report.json</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>nav</t>
+  </si>
+  <si>
+    <t>2026-09-29T20:27:01.361Z</t>
+  </si>
+  <si>
+    <t>http://127.0.0.1:8765/nav.html</t>
+  </si>
+  <si>
     <t>innovationlabgt/bronco.report.json</t>
   </si>
   <si>
@@ -67,7 +82,7 @@
     <t>innovationlabgt/bronco</t>
   </si>
   <si>
-    <t>2026-09-29T20:16:57.195Z</t>
+    <t>2026-09-29T20:46:25.964Z</t>
   </si>
 </sst>
 </file>
@@ -456,7 +471,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="36" customWidth="1"/>
@@ -534,15 +549,41 @@
         <v>11</v>
       </c>
       <c r="E3" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="F3" t="s">
         <v>18</v>
       </c>
       <c r="G3" t="s">
+        <v>17</v>
+      </c>
+      <c r="H3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E4" t="s">
+        <v>10</v>
+      </c>
+      <c r="F4" t="s">
+        <v>23</v>
+      </c>
+      <c r="G4" t="s">
         <v>13</v>
       </c>
-      <c r="H3" t="s">
+      <c r="H4" t="s">
         <v>14</v>
       </c>
     </row>

</xml_diff>